<commit_message>
Done login 001-017, TC015 fail do bug
</commit_message>
<xml_diff>
--- a/src/test/resources/Login_TC.xlsx
+++ b/src/test/resources/Login_TC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\automation-framework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E963ED1-0004-4663-AD82-CC47B3F55968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F2ACCE-9713-477C-AEA0-B2256484BF60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{014559CE-770C-44B1-B217-FE0B04801BDC}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1333" uniqueCount="422">
   <si>
     <t>Created Date: 20/05/2025</t>
   </si>
@@ -1096,12 +1096,6 @@
     <t>Value</t>
   </si>
   <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
     <t>chivq9@fpt.com</t>
   </si>
   <si>
@@ -1255,9 +1249,6 @@
     <t>loginwithmicrosoft</t>
   </si>
   <si>
-    <t>${email}|${password}</t>
-  </si>
-  <si>
     <t>SSO login</t>
   </si>
   <si>
@@ -1379,9 +1370,6 @@
   </si>
   <si>
     <t>Đăng nhập tài khoản đã có Mã Bảo mật - Kiểm tra Giới hạn nhập mã PIN</t>
-  </si>
-  <si>
-    <t>BE: Lỗi cộng dồn 5 lần nhập fail</t>
   </si>
   <si>
     <t>Đăng nhập tài khoản đã có Mã Bảo mật - Đăng nhập bằng SSO - Upload mã QR Pin thành công</t>
@@ -1592,12 +1580,6 @@
     <t>GLOBAL</t>
   </si>
   <si>
-    <t>passphrase</t>
-  </si>
-  <si>
-    <t>microsoftOtp</t>
-  </si>
-  <si>
     <t>Autotest send message PK-005</t>
   </si>
   <si>
@@ -1704,9 +1686,6 @@
     <t>Hội thoại|Tin nhắn|Chat|Chats|Conversation|Search|Message</t>
   </si>
   <si>
-    <t>${wrongPassphrase}</t>
-  </si>
-  <si>
     <t>Enter invalid passphrase</t>
   </si>
   <si>
@@ -1746,12 +1725,6 @@
     <t>Submit invalid PIN attempt 5</t>
   </si>
   <si>
-    <t>temporarily locked|tạm khóa|tạm khoá|vui lòng thử lại|5 attempts|attempts remaining</t>
-  </si>
-  <si>
-    <t>Account lock/attempt limit message should be displayed</t>
-  </si>
-  <si>
     <t>Switch to QR login screen</t>
   </si>
   <si>
@@ -1794,12 +1767,6 @@
     <t>Invalid QR upload attempt 5</t>
   </si>
   <si>
-    <t>temporarily locked|tạm khóa|tạm khoá|vui lòng thử lại|5 attempts|attempts remaining|QR Code  is incorrect, please try again!|QR Code is incorrect|please try again</t>
-  </si>
-  <si>
-    <t>QR upload limit/lock message should be displayed</t>
-  </si>
-  <si>
     <t>Open forgot code flow</t>
   </si>
   <si>
@@ -1824,65 +1791,161 @@
     <t>secure.qrInvalidPath</t>
   </si>
   <si>
-    <t>${secure.email}</t>
-  </si>
-  <si>
-    <t>${secure.password}</t>
+    <t>${secure.qrValidPath}</t>
+  </si>
+  <si>
+    <t>${secure.qrInvalidPath}</t>
+  </si>
+  <si>
+    <t>src\test\resources\QR login\Chivq9_UAT_QR.png</t>
+  </si>
+  <si>
+    <t>Fptchat@1234</t>
+  </si>
+  <si>
+    <t>nonSecure.email</t>
+  </si>
+  <si>
+    <t>nonSecure.password</t>
+  </si>
+  <si>
+    <t>fptchat01@fpt.com</t>
+  </si>
+  <si>
+    <t>Devteam@1234562</t>
+  </si>
+  <si>
+    <t>secure.InvalidPassphrase</t>
+  </si>
+  <si>
+    <t>Invalid@1234</t>
+  </si>
+  <si>
+    <t>${secure.InvalidPassphrase}</t>
+  </si>
+  <si>
+    <t>Skipped: message text assertion is more stable than SVG icon assertion</t>
+  </si>
+  <si>
+    <t>PIN code is incorrect|Pin code is incorrect|attempts remaining|incorrect|khÃ´ng Ä‘Ãºng|khÃ´ng há»£p lá»‡|MÃ£ báº£o máº­t</t>
+  </si>
+  <si>
+    <t>//button[@type='button' and (.//span[normalize-space()='Gửi' or normalize-space()='Send'] or normalize-space()='Gửi' or normalize-space()='Send')]</t>
+  </si>
+  <si>
+    <t>${nonSecure.email}|${nonSecure.password}</t>
+  </si>
+  <si>
+    <t>nonSecure.account</t>
+  </si>
+  <si>
+    <t>fptchat01</t>
+  </si>
+  <si>
+    <t>chivq9</t>
+  </si>
+  <si>
+    <t>${secure.email}|${secure.password}</t>
   </si>
   <si>
     <t>${secure.passphrase}</t>
   </si>
   <si>
-    <t>${secure.qrValidPath}</t>
-  </si>
-  <si>
-    <t>${secure.qrInvalidPath}</t>
-  </si>
-  <si>
-    <t>${nonSecure.account}</t>
-  </si>
-  <si>
-    <t>src\test\resources\QR login\Chivq9_UAT_QR.png</t>
-  </si>
-  <si>
-    <t>Fptchat@1234</t>
-  </si>
-  <si>
-    <t>nonSecure.email</t>
-  </si>
-  <si>
-    <t>nonSecure.password</t>
-  </si>
-  <si>
-    <t>fptchat01@fpt.com</t>
-  </si>
-  <si>
-    <t>Devteam@1234562</t>
-  </si>
-  <si>
-    <t>secure.InvalidPassphrase</t>
-  </si>
-  <si>
-    <t>Invalid@1234</t>
-  </si>
-  <si>
-    <t>${secure.InvalidPassphrase}</t>
-  </si>
-  <si>
-    <t>Skipped: message text assertion is more stable than SVG icon assertion</t>
-  </si>
-  <si>
-    <t>PIN code is incorrect|Pin code is incorrect|attempts remaining|incorrect|khÃ´ng Ä‘Ãºng|khÃ´ng há»£p lá»‡|MÃ£ báº£o máº­t</t>
-  </si>
-  <si>
-    <t>//button[@type='button' and (.//span[normalize-space()='Gửi' or normalize-space()='Send'] or normalize-space()='Gửi' or normalize-space()='Send')]</t>
+    <t>Ready</t>
+  </si>
+  <si>
+    <t>You have entered the wrong PIN too many times. Please try again in 60 minutes.</t>
+  </si>
+  <si>
+    <t>After exactly 5 invalid PIN submissions, lock message must be displayed</t>
+  </si>
+  <si>
+    <t>1 attempts remaining|1 attempt remaining</t>
+  </si>
+  <si>
+    <t>After invalid PIN attempt 4</t>
+  </si>
+  <si>
+    <t>2 attempts remaining</t>
+  </si>
+  <si>
+    <t>After invalid PIN attempt 3</t>
+  </si>
+  <si>
+    <t>3 attempts remaining</t>
+  </si>
+  <si>
+    <t>After invalid PIN attempt 2</t>
+  </si>
+  <si>
+    <t>4 attempts remaining</t>
+  </si>
+  <si>
+    <t>After invalid PIN attempt 1</t>
+  </si>
+  <si>
+    <t>Nhập sai mã PIN 5 lần, mỗi lần hiển thị số attempts remaining giảm dần 4 &gt; 3 &gt; 2 &gt; 1, sau lần thứ 5 hiển thị message khóa 60 phút.</t>
+  </si>
+  <si>
+    <t>Verify đúng sequence lỗi nhập sai PIN và message lock sau 5 lần</t>
+  </si>
+  <si>
+    <t>security.qrDeleteButton</t>
+  </si>
+  <si>
+    <t>(//*[local-name()='svg' and @viewBox='0 0 24 24' and .//*[local-name()='path' and contains(@d,'M16 8') and contains(@d,'L16 16')]]/ancestor::*[self::button or @role='button' or contains(@class,'cursor-pointer')][1] | //*[local-name()='svg' and @viewBox='0 0 24 24' and .//*[local-name()='path' and contains(@d,'M16 8') and contains(@d,'L16 16')]])[1]</t>
+  </si>
+  <si>
+    <t>QR error should be displayed after attempt 1</t>
+  </si>
+  <si>
+    <t>Delete invalid QR after attempt 1</t>
+  </si>
+  <si>
+    <t>QR error should be displayed after attempt 2</t>
+  </si>
+  <si>
+    <t>Delete invalid QR after attempt 2</t>
+  </si>
+  <si>
+    <t>QR error should be displayed after attempt 3</t>
+  </si>
+  <si>
+    <t>Delete invalid QR after attempt 3</t>
+  </si>
+  <si>
+    <t>QR error should be displayed after attempt 4</t>
+  </si>
+  <si>
+    <t>Delete invalid QR after attempt 4</t>
+  </si>
+  <si>
+    <t>QR error should be displayed after attempt 5</t>
+  </si>
+  <si>
+    <t>Delete invalid QR after attempt 5</t>
+  </si>
+  <si>
+    <t>Invalid QR upload attempt 6</t>
+  </si>
+  <si>
+    <t>Bạn đã nhập sai mã PIN quá số lần cho phép. Vui lòng thử lại sau</t>
+  </si>
+  <si>
+    <t>After attempt 6, QR PIN limit message should be displayed</t>
+  </si>
+  <si>
+    <t>Upload QR sai 5 lần: mỗi lần hiển thị lỗi QR và cho phép xóa ảnh để upload lại. Lần upload sai thứ 6 hiển thị message: Bạn đã nhập sai mã PIN quá số lần cho phép. Vui lòng thử lại sau</t>
+  </si>
+  <si>
+    <t>Verify giới hạn upload QR sai: xóa QR giữa các lần upload, lock ở lần thứ 6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1963,6 +2026,13 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2064,7 +2134,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2129,6 +2199,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2469,10 +2543,10 @@
         <v>175</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D1" s="22" t="s">
         <v>11</v>
@@ -2489,10 +2563,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C2" t="s">
-        <v>227</v>
+        <v>189</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
@@ -2501,7 +2575,7 @@
         <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2509,10 +2583,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C3" t="s">
-        <v>227</v>
+        <v>189</v>
       </c>
       <c r="D3" t="s">
         <v>19</v>
@@ -2521,7 +2595,7 @@
         <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2529,10 +2603,10 @@
         <v>20</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C4" t="s">
-        <v>227</v>
+        <v>189</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -2541,27 +2615,27 @@
         <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="26" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>226</v>
-      </c>
-      <c r="C5" t="s">
-        <v>227</v>
-      </c>
-      <c r="D5" t="s">
-        <v>185</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="B5" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
-        <v>228</v>
+      <c r="F5" s="26" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2569,10 +2643,10 @@
         <v>25</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C6" t="s">
-        <v>227</v>
+        <v>189</v>
       </c>
       <c r="D6" t="s">
         <v>27</v>
@@ -2581,46 +2655,46 @@
         <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="26" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="24" t="s">
-        <v>226</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B7" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="26" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="27" t="s">
         <v>227</v>
       </c>
-      <c r="D7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="C8" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="F7" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>230</v>
-      </c>
-      <c r="C8" t="s">
-        <v>227</v>
-      </c>
-      <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="F8" s="26" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2629,36 +2703,36 @@
         <v>35</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="10" spans="1:6" s="26" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="24" t="s">
-        <v>232</v>
-      </c>
-      <c r="C10" t="s">
-        <v>227</v>
-      </c>
-      <c r="D10" s="24" t="s">
+      <c r="B10" s="27" t="s">
+        <v>229</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="D10" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="F10" t="s">
-        <v>189</v>
+      <c r="F10" s="26" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -2666,10 +2740,10 @@
         <v>43</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C11" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>45</v>
@@ -2678,7 +2752,7 @@
         <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -2686,10 +2760,10 @@
         <v>46</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D12" s="24" t="s">
         <v>48</v>
@@ -2698,27 +2772,27 @@
         <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="26" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="24" t="s">
-        <v>235</v>
-      </c>
-      <c r="C13" t="s">
-        <v>227</v>
-      </c>
-      <c r="D13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" t="s">
-        <v>236</v>
+      <c r="B13" s="27" t="s">
+        <v>232</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>403</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -2726,10 +2800,10 @@
         <v>54</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C14" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D14" s="24" t="s">
         <v>56</v>
@@ -2746,10 +2820,10 @@
         <v>58</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C15" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>60</v>
@@ -2758,38 +2832,38 @@
         <v>52</v>
       </c>
       <c r="F15" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="26" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="24" t="s">
-        <v>240</v>
-      </c>
-      <c r="C16" t="s">
-        <v>227</v>
-      </c>
-      <c r="D16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B16" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>420</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>65</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="C17" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D17" s="24" t="s">
         <v>66</v>
@@ -2798,27 +2872,27 @@
         <v>17</v>
       </c>
       <c r="F17" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>67</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C18" t="s">
-        <v>227</v>
-      </c>
-      <c r="D18" t="s">
+        <v>189</v>
+      </c>
+      <c r="D18" s="24" t="s">
         <v>70</v>
       </c>
       <c r="E18" t="s">
         <v>17</v>
       </c>
       <c r="F18" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2826,10 +2900,10 @@
         <v>71</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="C19" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D19" t="s">
         <v>73</v>
@@ -2838,7 +2912,7 @@
         <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -2846,10 +2920,10 @@
         <v>74</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C20" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D20" t="s">
         <v>76</v>
@@ -2866,10 +2940,10 @@
         <v>77</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C21" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D21" t="s">
         <v>79</v>
@@ -2886,10 +2960,10 @@
         <v>80</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C22" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D22" t="s">
         <v>82</v>
@@ -2898,7 +2972,7 @@
         <v>17</v>
       </c>
       <c r="F22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2906,19 +2980,19 @@
         <v>83</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C23" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D23" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E23" t="s">
         <v>23</v>
       </c>
       <c r="F23" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2926,10 +3000,10 @@
         <v>87</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="C24" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D24" t="s">
         <v>89</v>
@@ -2938,7 +3012,7 @@
         <v>52</v>
       </c>
       <c r="F24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2946,10 +3020,10 @@
         <v>91</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="C25" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D25" t="s">
         <v>94</v>
@@ -2958,7 +3032,7 @@
         <v>17</v>
       </c>
       <c r="F25" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -2966,10 +3040,10 @@
         <v>95</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C26" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D26" t="s">
         <v>97</v>
@@ -2978,7 +3052,7 @@
         <v>17</v>
       </c>
       <c r="F26" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -2986,10 +3060,10 @@
         <v>98</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="C27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D27" t="s">
         <v>100</v>
@@ -2998,7 +3072,7 @@
         <v>17</v>
       </c>
       <c r="F27" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -3006,10 +3080,10 @@
         <v>101</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C28" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D28" t="s">
         <v>104</v>
@@ -3018,7 +3092,7 @@
         <v>17</v>
       </c>
       <c r="F28" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -3026,10 +3100,10 @@
         <v>105</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C29" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D29" t="s">
         <v>104</v>
@@ -3038,7 +3112,7 @@
         <v>17</v>
       </c>
       <c r="F29" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -3046,10 +3120,10 @@
         <v>107</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C30" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D30" t="s">
         <v>104</v>
@@ -3058,7 +3132,7 @@
         <v>17</v>
       </c>
       <c r="F30" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3066,10 +3140,10 @@
         <v>109</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C31" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D31" t="s">
         <v>112</v>
@@ -3078,7 +3152,7 @@
         <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3086,10 +3160,10 @@
         <v>113</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C32" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D32" t="s">
         <v>115</v>
@@ -3098,7 +3172,7 @@
         <v>17</v>
       </c>
       <c r="F32" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3106,10 +3180,10 @@
         <v>116</v>
       </c>
       <c r="B33" s="24" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C33" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D33" t="s">
         <v>118</v>
@@ -3118,7 +3192,7 @@
         <v>23</v>
       </c>
       <c r="F33" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3126,10 +3200,10 @@
         <v>119</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C34" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D34" t="s">
         <v>121</v>
@@ -3138,7 +3212,7 @@
         <v>23</v>
       </c>
       <c r="F34" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3146,10 +3220,10 @@
         <v>122</v>
       </c>
       <c r="B35" s="24" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C35" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D35" t="s">
         <v>125</v>
@@ -3166,10 +3240,10 @@
         <v>126</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C36" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D36" t="s">
         <v>128</v>
@@ -3178,7 +3252,7 @@
         <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3186,10 +3260,10 @@
         <v>129</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="C37" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D37" t="s">
         <v>131</v>
@@ -3198,7 +3272,7 @@
         <v>23</v>
       </c>
       <c r="F37" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3206,10 +3280,10 @@
         <v>132</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C38" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D38" t="s">
         <v>135</v>
@@ -3218,7 +3292,7 @@
         <v>17</v>
       </c>
       <c r="F38" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -3226,10 +3300,10 @@
         <v>136</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C39" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D39" t="s">
         <v>138</v>
@@ -3238,7 +3312,7 @@
         <v>17</v>
       </c>
       <c r="F39" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3246,10 +3320,10 @@
         <v>139</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C40" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D40" t="s">
         <v>141</v>
@@ -3258,7 +3332,7 @@
         <v>17</v>
       </c>
       <c r="F40" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -3266,10 +3340,10 @@
         <v>142</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="C41" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D41" t="s">
         <v>145</v>
@@ -3278,7 +3352,7 @@
         <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -3286,10 +3360,10 @@
         <v>146</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C42" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D42" t="s">
         <v>148</v>
@@ -3298,7 +3372,7 @@
         <v>42</v>
       </c>
       <c r="F42" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -3306,19 +3380,19 @@
         <v>149</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C43" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D43" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="E43" t="s">
         <v>17</v>
       </c>
       <c r="F43" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -3326,10 +3400,10 @@
         <v>153</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C44" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D44" t="s">
         <v>76</v>
@@ -3346,10 +3420,10 @@
         <v>155</v>
       </c>
       <c r="B45" s="24" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C45" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D45" t="s">
         <v>157</v>
@@ -3358,7 +3432,7 @@
         <v>17</v>
       </c>
       <c r="F45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -3366,10 +3440,10 @@
         <v>158</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C46" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D46" t="s">
         <v>161</v>
@@ -3378,7 +3452,7 @@
         <v>17</v>
       </c>
       <c r="F46" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3386,10 +3460,10 @@
         <v>162</v>
       </c>
       <c r="B47" s="24" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="C47" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D47" t="s">
         <v>161</v>
@@ -3406,10 +3480,10 @@
         <v>165</v>
       </c>
       <c r="B48" s="24" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="C48" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D48" t="s">
         <v>161</v>
@@ -3418,7 +3492,7 @@
         <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -3426,19 +3500,19 @@
         <v>167</v>
       </c>
       <c r="B49" s="24" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="C49" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D49" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="E49" t="s">
         <v>52</v>
       </c>
       <c r="F49" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -3446,30 +3520,31 @@
         <v>172</v>
       </c>
       <c r="B50" s="24" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C50" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D50" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="E50" t="s">
         <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="C1:C50" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -3485,19 +3560,19 @@
         <v>175</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -3505,19 +3580,19 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D2" t="s">
         <v>188</v>
       </c>
-      <c r="C2" t="s">
-        <v>189</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>189</v>
+      </c>
+      <c r="F2" t="s">
         <v>190</v>
-      </c>
-      <c r="E2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F2" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3525,19 +3600,19 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D3" t="s">
-        <v>194</v>
+        <v>386</v>
       </c>
       <c r="E3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3545,19 +3620,19 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E4" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3565,19 +3640,19 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F5" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3585,19 +3660,19 @@
         <v>18</v>
       </c>
       <c r="B6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" t="s">
         <v>188</v>
       </c>
-      <c r="C6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" t="s">
         <v>190</v>
-      </c>
-      <c r="E6" t="s">
-        <v>191</v>
-      </c>
-      <c r="F6" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -3605,19 +3680,19 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D7" t="s">
-        <v>194</v>
+        <v>386</v>
       </c>
       <c r="E7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -3625,19 +3700,19 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D8" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F8" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -3645,19 +3720,19 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F9" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -3665,19 +3740,19 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D10" t="s">
         <v>199</v>
       </c>
-      <c r="C10" t="s">
-        <v>189</v>
-      </c>
-      <c r="D10" t="s">
-        <v>202</v>
-      </c>
       <c r="E10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F10" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -3685,19 +3760,19 @@
         <v>25</v>
       </c>
       <c r="B11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" t="s">
+        <v>187</v>
+      </c>
+      <c r="D11" t="s">
         <v>188</v>
       </c>
-      <c r="C11" t="s">
-        <v>189</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>189</v>
+      </c>
+      <c r="F11" t="s">
         <v>190</v>
-      </c>
-      <c r="E11" t="s">
-        <v>191</v>
-      </c>
-      <c r="F11" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -3705,19 +3780,19 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D12" t="s">
-        <v>194</v>
+        <v>386</v>
       </c>
       <c r="E12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F12" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -3725,19 +3800,19 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D13" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E13" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -3745,19 +3820,19 @@
         <v>25</v>
       </c>
       <c r="B14" t="s">
+        <v>201</v>
+      </c>
+      <c r="C14" t="s">
+        <v>187</v>
+      </c>
+      <c r="D14" t="s">
+        <v>187</v>
+      </c>
+      <c r="E14" t="s">
+        <v>189</v>
+      </c>
+      <c r="F14" t="s">
         <v>204</v>
-      </c>
-      <c r="C14" t="s">
-        <v>189</v>
-      </c>
-      <c r="D14" t="s">
-        <v>189</v>
-      </c>
-      <c r="E14" t="s">
-        <v>191</v>
-      </c>
-      <c r="F14" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -3765,19 +3840,19 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C15" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D15" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E15" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F15" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -3785,19 +3860,19 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D16" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E16" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F16" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -3805,19 +3880,19 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C17" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E17" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F17" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -3825,19 +3900,19 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
+        <v>186</v>
+      </c>
+      <c r="C18" t="s">
+        <v>187</v>
+      </c>
+      <c r="D18" t="s">
         <v>188</v>
       </c>
-      <c r="C18" t="s">
-        <v>189</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>189</v>
+      </c>
+      <c r="F18" t="s">
         <v>190</v>
-      </c>
-      <c r="E18" t="s">
-        <v>191</v>
-      </c>
-      <c r="F18" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -3845,19 +3920,19 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D19" t="s">
-        <v>194</v>
+        <v>386</v>
       </c>
       <c r="E19" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F19" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -3865,19 +3940,19 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C20" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D20" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E20" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F20" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -3885,19 +3960,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>201</v>
+      </c>
+      <c r="C21" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21" t="s">
+        <v>187</v>
+      </c>
+      <c r="E21" t="s">
+        <v>189</v>
+      </c>
+      <c r="F21" t="s">
         <v>204</v>
-      </c>
-      <c r="C21" t="s">
-        <v>189</v>
-      </c>
-      <c r="D21" t="s">
-        <v>189</v>
-      </c>
-      <c r="E21" t="s">
-        <v>191</v>
-      </c>
-      <c r="F21" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -3905,19 +3980,19 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E22" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F22" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -3925,19 +4000,19 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C23" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D23" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E23" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -3945,19 +4020,19 @@
         <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D24" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E24" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F24" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -3965,19 +4040,19 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
+        <v>186</v>
+      </c>
+      <c r="C25" t="s">
+        <v>187</v>
+      </c>
+      <c r="D25" t="s">
         <v>188</v>
       </c>
-      <c r="C25" t="s">
-        <v>189</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
+        <v>189</v>
+      </c>
+      <c r="F25" t="s">
         <v>190</v>
-      </c>
-      <c r="E25" t="s">
-        <v>191</v>
-      </c>
-      <c r="F25" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -3985,19 +4060,19 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C26" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D26" t="s">
-        <v>194</v>
+        <v>390</v>
       </c>
       <c r="E26" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F26" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -4005,19 +4080,19 @@
         <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C27" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D27" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E27" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F27" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -4025,19 +4100,19 @@
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="C28" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D28" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E28" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F28" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -4045,19 +4120,19 @@
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D29" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="E29" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F29" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -4065,19 +4140,19 @@
         <v>43</v>
       </c>
       <c r="B30" t="s">
+        <v>186</v>
+      </c>
+      <c r="C30" t="s">
+        <v>187</v>
+      </c>
+      <c r="D30" t="s">
         <v>188</v>
       </c>
-      <c r="C30" t="s">
-        <v>189</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
+        <v>189</v>
+      </c>
+      <c r="F30" t="s">
         <v>190</v>
-      </c>
-      <c r="E30" t="s">
-        <v>191</v>
-      </c>
-      <c r="F30" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -4085,19 +4160,19 @@
         <v>43</v>
       </c>
       <c r="B31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C31" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D31" t="s">
-        <v>194</v>
+        <v>390</v>
       </c>
       <c r="E31" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F31" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -4105,19 +4180,19 @@
         <v>43</v>
       </c>
       <c r="B32" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C32" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D32" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E32" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F32" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -4125,19 +4200,19 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C33" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D33" t="s">
-        <v>337</v>
+        <v>391</v>
       </c>
       <c r="E33" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F33" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -4145,19 +4220,19 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C34" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D34" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="E34" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F34" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -4165,19 +4240,19 @@
         <v>43</v>
       </c>
       <c r="B35" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C35" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D35" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="E35" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F35" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -4185,19 +4260,19 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
+        <v>186</v>
+      </c>
+      <c r="C36" t="s">
+        <v>187</v>
+      </c>
+      <c r="D36" t="s">
         <v>188</v>
       </c>
-      <c r="C36" t="s">
-        <v>189</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
+        <v>189</v>
+      </c>
+      <c r="F36" t="s">
         <v>190</v>
-      </c>
-      <c r="E36" t="s">
-        <v>191</v>
-      </c>
-      <c r="F36" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -4205,19 +4280,19 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C37" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D37" t="s">
-        <v>194</v>
+        <v>390</v>
       </c>
       <c r="E37" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F37" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -4225,19 +4300,19 @@
         <v>46</v>
       </c>
       <c r="B38" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C38" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D38" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E38" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F38" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -4245,19 +4320,19 @@
         <v>46</v>
       </c>
       <c r="B39" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C39" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D39" t="s">
-        <v>397</v>
+        <v>382</v>
       </c>
       <c r="E39" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F39" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -4265,19 +4340,19 @@
         <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C40" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D40" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="E40" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F40" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -4285,19 +4360,19 @@
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="C41" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="D41" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E41" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F41" t="s">
-        <v>398</v>
+        <v>383</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -4305,19 +4380,19 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C42" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D42" t="s">
-        <v>399</v>
+        <v>384</v>
       </c>
       <c r="E42" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F42" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -4325,19 +4400,19 @@
         <v>49</v>
       </c>
       <c r="B43" t="s">
+        <v>186</v>
+      </c>
+      <c r="C43" t="s">
+        <v>187</v>
+      </c>
+      <c r="D43" t="s">
         <v>188</v>
       </c>
-      <c r="C43" t="s">
-        <v>189</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
+        <v>189</v>
+      </c>
+      <c r="F43" t="s">
         <v>190</v>
-      </c>
-      <c r="E43" t="s">
-        <v>191</v>
-      </c>
-      <c r="F43" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -4345,19 +4420,19 @@
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C44" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D44" t="s">
-        <v>194</v>
+        <v>390</v>
       </c>
       <c r="E44" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F44" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -4365,19 +4440,19 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D45" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E45" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F45" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -4385,19 +4460,19 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C46" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D46" t="s">
-        <v>343</v>
+        <v>382</v>
       </c>
       <c r="E46" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F46" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -4405,19 +4480,19 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C47" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D47" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="E47" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F47" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -4425,19 +4500,16 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>336</v>
-      </c>
-      <c r="C48" t="s">
-        <v>317</v>
+        <v>196</v>
       </c>
       <c r="D48" t="s">
-        <v>343</v>
+        <v>401</v>
       </c>
       <c r="E48" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F48" t="s">
-        <v>349</v>
+        <v>402</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -4445,19 +4517,19 @@
         <v>49</v>
       </c>
       <c r="B49" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="C49" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="D49" t="s">
-        <v>340</v>
+        <v>382</v>
       </c>
       <c r="E49" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F49" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -4465,19 +4537,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C50" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D50" t="s">
+        <v>334</v>
+      </c>
+      <c r="E50" t="s">
+        <v>189</v>
+      </c>
+      <c r="F50" t="s">
         <v>343</v>
-      </c>
-      <c r="E50" t="s">
-        <v>191</v>
-      </c>
-      <c r="F50" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -4485,19 +4557,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>339</v>
-      </c>
-      <c r="C51" t="s">
-        <v>319</v>
+        <v>196</v>
       </c>
       <c r="D51" t="s">
-        <v>340</v>
+        <v>399</v>
       </c>
       <c r="E51" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F51" t="s">
-        <v>352</v>
+        <v>400</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -4505,19 +4574,19 @@
         <v>49</v>
       </c>
       <c r="B52" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C52" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D52" t="s">
-        <v>343</v>
+        <v>382</v>
       </c>
       <c r="E52" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F52" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -4525,19 +4594,19 @@
         <v>49</v>
       </c>
       <c r="B53" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C53" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D53" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="E53" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F53" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -4545,19 +4614,16 @@
         <v>49</v>
       </c>
       <c r="B54" t="s">
-        <v>336</v>
-      </c>
-      <c r="C54" t="s">
-        <v>317</v>
+        <v>196</v>
       </c>
       <c r="D54" t="s">
-        <v>343</v>
+        <v>397</v>
       </c>
       <c r="E54" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F54" t="s">
-        <v>355</v>
+        <v>398</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -4565,19 +4631,19 @@
         <v>49</v>
       </c>
       <c r="B55" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="C55" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="D55" t="s">
-        <v>340</v>
+        <v>382</v>
       </c>
       <c r="E55" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F55" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -4585,99 +4651,96 @@
         <v>49</v>
       </c>
       <c r="B56" t="s">
-        <v>199</v>
+        <v>333</v>
       </c>
       <c r="C56" t="s">
-        <v>189</v>
+        <v>313</v>
       </c>
       <c r="D56" t="s">
-        <v>357</v>
+        <v>334</v>
       </c>
       <c r="E56" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F56" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B57" t="s">
-        <v>188</v>
-      </c>
-      <c r="C57" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D57" t="s">
-        <v>190</v>
+        <v>395</v>
       </c>
       <c r="E57" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F57" t="s">
-        <v>192</v>
+        <v>396</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B58" t="s">
-        <v>193</v>
+        <v>330</v>
       </c>
       <c r="C58" t="s">
-        <v>189</v>
+        <v>311</v>
       </c>
       <c r="D58" t="s">
-        <v>194</v>
+        <v>382</v>
       </c>
       <c r="E58" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F58" t="s">
-        <v>195</v>
+        <v>348</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B59" t="s">
-        <v>196</v>
+        <v>333</v>
       </c>
       <c r="C59" t="s">
-        <v>189</v>
+        <v>313</v>
       </c>
       <c r="D59" t="s">
-        <v>197</v>
+        <v>334</v>
       </c>
       <c r="E59" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F59" t="s">
-        <v>198</v>
+        <v>349</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B60" t="s">
-        <v>339</v>
+        <v>196</v>
       </c>
       <c r="C60" t="s">
-        <v>320</v>
+        <v>187</v>
       </c>
       <c r="D60" t="s">
-        <v>340</v>
+        <v>393</v>
       </c>
       <c r="E60" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F60" t="s">
-        <v>359</v>
+        <v>394</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -4685,19 +4748,19 @@
         <v>54</v>
       </c>
       <c r="B61" t="s">
-        <v>360</v>
+        <v>186</v>
       </c>
       <c r="C61" t="s">
-        <v>322</v>
+        <v>187</v>
       </c>
       <c r="D61" t="s">
-        <v>361</v>
+        <v>188</v>
       </c>
       <c r="E61" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F61" t="s">
-        <v>362</v>
+        <v>190</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -4705,99 +4768,99 @@
         <v>54</v>
       </c>
       <c r="B62" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C62" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D62" t="s">
-        <v>342</v>
+        <v>390</v>
       </c>
       <c r="E62" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F62" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B63" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C63" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D63" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E63" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F63" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B64" t="s">
-        <v>193</v>
+        <v>333</v>
       </c>
       <c r="C64" t="s">
-        <v>189</v>
+        <v>314</v>
       </c>
       <c r="D64" t="s">
-        <v>194</v>
+        <v>334</v>
       </c>
       <c r="E64" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F64" t="s">
-        <v>195</v>
+        <v>350</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B65" t="s">
-        <v>196</v>
+        <v>351</v>
       </c>
       <c r="C65" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="D65" t="s">
-        <v>197</v>
+        <v>352</v>
       </c>
       <c r="E65" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F65" t="s">
-        <v>198</v>
+        <v>353</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B66" t="s">
-        <v>339</v>
+        <v>196</v>
       </c>
       <c r="C66" t="s">
-        <v>320</v>
+        <v>187</v>
       </c>
       <c r="D66" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E66" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F66" t="s">
-        <v>359</v>
+        <v>200</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
@@ -4805,19 +4868,19 @@
         <v>58</v>
       </c>
       <c r="B67" t="s">
-        <v>360</v>
+        <v>186</v>
       </c>
       <c r="C67" t="s">
-        <v>322</v>
+        <v>187</v>
       </c>
       <c r="D67" t="s">
-        <v>363</v>
+        <v>188</v>
       </c>
       <c r="E67" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F67" t="s">
-        <v>364</v>
+        <v>190</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -4825,19 +4888,19 @@
         <v>58</v>
       </c>
       <c r="B68" t="s">
-        <v>332</v>
+        <v>191</v>
       </c>
       <c r="C68" t="s">
-        <v>326</v>
+        <v>187</v>
       </c>
       <c r="D68" t="s">
-        <v>189</v>
+        <v>390</v>
       </c>
       <c r="E68" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F68" t="s">
-        <v>365</v>
+        <v>192</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -4845,99 +4908,99 @@
         <v>58</v>
       </c>
       <c r="B69" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C69" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D69" t="s">
-        <v>366</v>
+        <v>194</v>
       </c>
       <c r="E69" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F69" t="s">
-        <v>367</v>
+        <v>195</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B70" t="s">
-        <v>188</v>
+        <v>333</v>
       </c>
       <c r="C70" t="s">
-        <v>189</v>
+        <v>314</v>
       </c>
       <c r="D70" t="s">
-        <v>190</v>
+        <v>334</v>
       </c>
       <c r="E70" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F70" t="s">
-        <v>192</v>
+        <v>350</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B71" t="s">
-        <v>193</v>
+        <v>351</v>
       </c>
       <c r="C71" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="D71" t="s">
-        <v>194</v>
+        <v>354</v>
       </c>
       <c r="E71" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F71" t="s">
-        <v>195</v>
+        <v>355</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B72" t="s">
-        <v>196</v>
+        <v>326</v>
       </c>
       <c r="C72" t="s">
-        <v>189</v>
+        <v>320</v>
       </c>
       <c r="D72" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="E72" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F72" t="s">
-        <v>198</v>
+        <v>356</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B73" t="s">
-        <v>339</v>
+        <v>196</v>
       </c>
       <c r="C73" t="s">
-        <v>320</v>
+        <v>187</v>
       </c>
       <c r="D73" t="s">
-        <v>340</v>
+        <v>357</v>
       </c>
       <c r="E73" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F73" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -4945,19 +5008,16 @@
         <v>62</v>
       </c>
       <c r="B74" t="s">
-        <v>360</v>
-      </c>
-      <c r="C74" t="s">
-        <v>322</v>
+        <v>186</v>
       </c>
       <c r="D74" t="s">
-        <v>363</v>
+        <v>188</v>
       </c>
       <c r="E74" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F74" t="s">
-        <v>368</v>
+        <v>190</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
@@ -4965,19 +5025,16 @@
         <v>62</v>
       </c>
       <c r="B75" t="s">
-        <v>360</v>
-      </c>
-      <c r="C75" t="s">
-        <v>322</v>
+        <v>191</v>
       </c>
       <c r="D75" t="s">
-        <v>363</v>
+        <v>390</v>
       </c>
       <c r="E75" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F75" t="s">
-        <v>369</v>
+        <v>192</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
@@ -4985,19 +5042,16 @@
         <v>62</v>
       </c>
       <c r="B76" t="s">
-        <v>360</v>
-      </c>
-      <c r="C76" t="s">
-        <v>322</v>
+        <v>193</v>
       </c>
       <c r="D76" t="s">
-        <v>363</v>
+        <v>194</v>
       </c>
       <c r="E76" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F76" t="s">
-        <v>370</v>
+        <v>195</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
@@ -5005,19 +5059,19 @@
         <v>62</v>
       </c>
       <c r="B77" t="s">
-        <v>360</v>
+        <v>333</v>
       </c>
       <c r="C77" t="s">
-        <v>322</v>
-      </c>
-      <c r="D77" t="s">
-        <v>363</v>
+        <v>314</v>
+      </c>
+      <c r="D77">
+        <v>10</v>
       </c>
       <c r="E77" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F77" t="s">
-        <v>371</v>
+        <v>350</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
@@ -5025,19 +5079,19 @@
         <v>62</v>
       </c>
       <c r="B78" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="C78" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="D78" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="E78" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F78" t="s">
-        <v>372</v>
+        <v>359</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
@@ -5045,179 +5099,461 @@
         <v>62</v>
       </c>
       <c r="B79" t="s">
-        <v>199</v>
-      </c>
-      <c r="C79" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D79" t="s">
-        <v>373</v>
+        <v>357</v>
       </c>
       <c r="E79" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F79" t="s">
-        <v>374</v>
+        <v>407</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B80" t="s">
-        <v>188</v>
+        <v>333</v>
       </c>
       <c r="C80" t="s">
-        <v>189</v>
-      </c>
-      <c r="D80" t="s">
-        <v>190</v>
+        <v>405</v>
+      </c>
+      <c r="D80">
+        <v>10</v>
       </c>
       <c r="E80" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F80" t="s">
-        <v>192</v>
+        <v>408</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B81" t="s">
-        <v>193</v>
+        <v>351</v>
       </c>
       <c r="C81" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="D81" t="s">
-        <v>194</v>
+        <v>354</v>
       </c>
       <c r="E81" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F81" t="s">
-        <v>195</v>
+        <v>360</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B82" t="s">
         <v>196</v>
       </c>
-      <c r="C82" t="s">
-        <v>189</v>
-      </c>
       <c r="D82" t="s">
-        <v>197</v>
+        <v>357</v>
       </c>
       <c r="E82" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F82" t="s">
-        <v>198</v>
+        <v>409</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B83" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C83" t="s">
-        <v>328</v>
-      </c>
-      <c r="D83" t="s">
-        <v>340</v>
+        <v>405</v>
+      </c>
+      <c r="D83">
+        <v>10</v>
       </c>
       <c r="E83" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F83" t="s">
-        <v>375</v>
+        <v>410</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B84" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="C84" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="D84" t="s">
-        <v>340</v>
+        <v>354</v>
       </c>
       <c r="E84" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F84" t="s">
-        <v>376</v>
+        <v>361</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B85" t="s">
-        <v>336</v>
-      </c>
-      <c r="C85" t="s">
-        <v>317</v>
+        <v>196</v>
       </c>
       <c r="D85" t="s">
-        <v>337</v>
+        <v>357</v>
       </c>
       <c r="E85" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F85" t="s">
-        <v>377</v>
+        <v>411</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B86" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C86" t="s">
-        <v>319</v>
-      </c>
-      <c r="D86" t="s">
-        <v>340</v>
+        <v>405</v>
+      </c>
+      <c r="D86">
+        <v>10</v>
       </c>
       <c r="E86" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F86" t="s">
-        <v>341</v>
+        <v>412</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
+        <v>62</v>
+      </c>
+      <c r="B87" t="s">
+        <v>351</v>
+      </c>
+      <c r="C87" t="s">
+        <v>316</v>
+      </c>
+      <c r="D87" t="s">
+        <v>354</v>
+      </c>
+      <c r="E87" t="s">
+        <v>189</v>
+      </c>
+      <c r="F87" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>62</v>
+      </c>
+      <c r="B88" t="s">
+        <v>196</v>
+      </c>
+      <c r="D88" t="s">
+        <v>357</v>
+      </c>
+      <c r="E88" t="s">
+        <v>189</v>
+      </c>
+      <c r="F88" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>62</v>
+      </c>
+      <c r="B89" t="s">
+        <v>333</v>
+      </c>
+      <c r="C89" t="s">
+        <v>405</v>
+      </c>
+      <c r="D89">
+        <v>10</v>
+      </c>
+      <c r="E89" t="s">
+        <v>189</v>
+      </c>
+      <c r="F89" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>62</v>
+      </c>
+      <c r="B90" t="s">
+        <v>351</v>
+      </c>
+      <c r="C90" t="s">
+        <v>316</v>
+      </c>
+      <c r="D90" t="s">
+        <v>354</v>
+      </c>
+      <c r="E90" t="s">
+        <v>189</v>
+      </c>
+      <c r="F90" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>62</v>
+      </c>
+      <c r="B91" t="s">
+        <v>196</v>
+      </c>
+      <c r="D91" t="s">
+        <v>357</v>
+      </c>
+      <c r="E91" t="s">
+        <v>189</v>
+      </c>
+      <c r="F91" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>62</v>
+      </c>
+      <c r="B92" t="s">
+        <v>333</v>
+      </c>
+      <c r="C92" t="s">
+        <v>405</v>
+      </c>
+      <c r="D92">
+        <v>10</v>
+      </c>
+      <c r="E92" t="s">
+        <v>189</v>
+      </c>
+      <c r="F92" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>62</v>
+      </c>
+      <c r="B93" t="s">
+        <v>351</v>
+      </c>
+      <c r="C93" t="s">
+        <v>316</v>
+      </c>
+      <c r="D93" t="s">
+        <v>354</v>
+      </c>
+      <c r="E93" t="s">
+        <v>189</v>
+      </c>
+      <c r="F93" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>62</v>
+      </c>
+      <c r="B94" t="s">
+        <v>196</v>
+      </c>
+      <c r="D94" t="s">
+        <v>418</v>
+      </c>
+      <c r="E94" t="s">
+        <v>189</v>
+      </c>
+      <c r="F94" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
         <v>65</v>
       </c>
-      <c r="B87" t="s">
-        <v>199</v>
-      </c>
-      <c r="C87" t="s">
-        <v>189</v>
-      </c>
-      <c r="D87" t="s">
-        <v>342</v>
-      </c>
-      <c r="E87" t="s">
+      <c r="B95" t="s">
+        <v>186</v>
+      </c>
+      <c r="C95" t="s">
+        <v>187</v>
+      </c>
+      <c r="D95" t="s">
+        <v>188</v>
+      </c>
+      <c r="E95" t="s">
+        <v>189</v>
+      </c>
+      <c r="F95" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>65</v>
+      </c>
+      <c r="B96" t="s">
         <v>191</v>
       </c>
-      <c r="F87" t="s">
-        <v>203</v>
+      <c r="C96" t="s">
+        <v>187</v>
+      </c>
+      <c r="D96" t="s">
+        <v>390</v>
+      </c>
+      <c r="E96" t="s">
+        <v>189</v>
+      </c>
+      <c r="F96" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>65</v>
+      </c>
+      <c r="B97" t="s">
+        <v>193</v>
+      </c>
+      <c r="C97" t="s">
+        <v>187</v>
+      </c>
+      <c r="D97" t="s">
+        <v>194</v>
+      </c>
+      <c r="E97" t="s">
+        <v>189</v>
+      </c>
+      <c r="F97" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>65</v>
+      </c>
+      <c r="B98" t="s">
+        <v>333</v>
+      </c>
+      <c r="C98" t="s">
+        <v>322</v>
+      </c>
+      <c r="D98" t="s">
+        <v>334</v>
+      </c>
+      <c r="E98" t="s">
+        <v>189</v>
+      </c>
+      <c r="F98" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>65</v>
+      </c>
+      <c r="B99" t="s">
+        <v>333</v>
+      </c>
+      <c r="C99" t="s">
+        <v>324</v>
+      </c>
+      <c r="D99" t="s">
+        <v>334</v>
+      </c>
+      <c r="E99" t="s">
+        <v>189</v>
+      </c>
+      <c r="F99" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>65</v>
+      </c>
+      <c r="B100" t="s">
+        <v>330</v>
+      </c>
+      <c r="C100" t="s">
+        <v>311</v>
+      </c>
+      <c r="D100" t="s">
+        <v>331</v>
+      </c>
+      <c r="E100" t="s">
+        <v>189</v>
+      </c>
+      <c r="F100" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>65</v>
+      </c>
+      <c r="B101" t="s">
+        <v>333</v>
+      </c>
+      <c r="C101" t="s">
+        <v>313</v>
+      </c>
+      <c r="D101" t="s">
+        <v>334</v>
+      </c>
+      <c r="E101" t="s">
+        <v>189</v>
+      </c>
+      <c r="F101" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>65</v>
+      </c>
+      <c r="B102" t="s">
+        <v>196</v>
+      </c>
+      <c r="C102" t="s">
+        <v>187</v>
+      </c>
+      <c r="D102" t="s">
+        <v>336</v>
+      </c>
+      <c r="E102" t="s">
+        <v>189</v>
+      </c>
+      <c r="F102" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5227,7 +5563,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -5240,7 +5576,7 @@
         <v>175</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C1" s="22" t="s">
         <v>176</v>
@@ -5248,189 +5584,156 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>305</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>177</v>
+        <v>202</v>
       </c>
       <c r="C2" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>305</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="C3" t="s">
-        <v>384</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B4" t="s">
         <v>306</v>
       </c>
       <c r="C4" t="s">
-        <v>385</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C5" t="s">
-        <v>189</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>301</v>
       </c>
       <c r="B6" t="s">
-        <v>205</v>
+        <v>309</v>
       </c>
       <c r="C6" t="s">
-        <v>388</v>
+        <v>373</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>301</v>
       </c>
       <c r="B7" t="s">
-        <v>206</v>
+        <v>367</v>
       </c>
       <c r="C7" t="s">
-        <v>308</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B8" t="s">
-        <v>312</v>
+        <v>368</v>
       </c>
       <c r="C8" t="s">
-        <v>313</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B9" t="s">
-        <v>314</v>
-      </c>
-      <c r="C9" t="s">
-        <v>386</v>
+        <v>369</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B10" t="s">
-        <v>315</v>
-      </c>
-      <c r="C10" t="s">
-        <v>387</v>
+        <v>380</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B11" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="C11" t="s">
-        <v>179</v>
+        <v>374</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B12" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="C12" t="s">
-        <v>180</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B13" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B14" t="s">
-        <v>395</v>
+        <v>377</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>396</v>
+        <v>379</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B15" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C15" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>305</v>
-      </c>
-      <c r="B16" t="s">
-        <v>382</v>
-      </c>
-      <c r="C16" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>305</v>
-      </c>
-      <c r="B17" t="s">
-        <v>391</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>305</v>
-      </c>
-      <c r="B18" t="s">
-        <v>392</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -5441,7 +5744,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
@@ -5451,189 +5754,200 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="22" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B2" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B3" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C3" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B4" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C4" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B5" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" t="s">
         <v>291</v>
-      </c>
-      <c r="C5" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C6" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B7" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C7" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B8" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C8" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B9" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C9" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="B10" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C10" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="B11" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C11" t="s">
-        <v>400</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B12" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C12" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="B13" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C13" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B14" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C14" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="B15" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C15" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C16" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="B17" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C17" t="s">
-        <v>331</v>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>405</v>
+      </c>
+      <c r="B18" t="s">
+        <v>287</v>
+      </c>
+      <c r="C18" t="s">
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -5662,10 +5976,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
@@ -5694,10 +6008,10 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="27"/>
+      <c r="B2" s="29"/>
       <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
@@ -5723,11 +6037,11 @@
       <c r="I2" s="17"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="27"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
@@ -5786,7 +6100,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>16</v>
@@ -5809,7 +6123,7 @@
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>19</v>
@@ -5832,7 +6146,7 @@
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>21</v>
@@ -5855,10 +6169,10 @@
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>23</v>
@@ -5958,7 +6272,7 @@
         <v>37</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>17</v>
@@ -6149,7 +6463,7 @@
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
create TestSuite and ActionKeywords sheet for tester
</commit_message>
<xml_diff>
--- a/src/test/resources/Login_TC.xlsx
+++ b/src/test/resources/Login_TC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\automation-framework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D442CC57-46D6-4E79-918A-C49F8178BF35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3F4CDE-8361-4BAF-82AD-F62F409E5C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{014559CE-770C-44B1-B217-FE0B04801BDC}"/>
   </bookViews>
@@ -1995,9 +1995,6 @@
     <t>idSubmit_SAOTCC_Continue</t>
   </si>
   <si>
-    <t>//*[@id='acceptButton' or @id='idSIButton9' or @value='Yes' or normalize-space(.)='Yes']</t>
-  </si>
-  <si>
     <t>//*[@id='root']//input | //button[.//span[normalize-space(.)='Bỏ qua'] or normalize-space(.)='Bỏ qua'] | //*[@data-placeholder='Search' or @data-placeholder='Message'] | //button[contains(@class,'send-btn')] | //span[contains(concat(' ',normalize-space(@class),' '),' slider ')]</t>
   </si>
   <si>
@@ -2044,6 +2041,9 @@
   </si>
   <si>
     <t>//*[contains(@class,'create-room') or contains(@class,'send-btn')] | //*[@data-placeholder='Search' or @data-placeholder='Message' or @data-placeholder='Tìm kiếm' or @data-placeholder='Tin nhắn'] | //*[@placeholder='Search' or @placeholder='Message' or @placeholder='Tìm kiếm' or @placeholder='Tin nhắn'] | //*[@aria-label='Search' or @aria-label='Message' or @aria-label='Tìm kiếm' or @aria-label='Tin nhắn']</t>
+  </si>
+  <si>
+    <t>//*[@id='acceptButton' or @id='idSIButton9' or @value='Yes' or @aria-label='Yes' or @title='Yes' or normalize-space(.)='Yes']</t>
   </si>
 </sst>
 </file>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D2" s="27"/>
       <c r="E2" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F2" s="27"/>
       <c r="G2" s="27"/>
@@ -3810,7 +3810,7 @@
         <v>405</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F5" s="27"/>
       <c r="G5" s="27"/>
@@ -3854,7 +3854,7 @@
         <v>410</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F7" s="27"/>
       <c r="G7" s="27"/>
@@ -3898,7 +3898,7 @@
         <v>413</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F9" s="27"/>
       <c r="G9" s="27"/>
@@ -3920,7 +3920,7 @@
         <v>416</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F10" s="27"/>
       <c r="G10" s="27"/>
@@ -3942,7 +3942,7 @@
         <v>418</v>
       </c>
       <c r="E11" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F11" s="27"/>
       <c r="G11" s="27"/>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="D14" s="27"/>
       <c r="E14" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F14" s="27"/>
       <c r="G14" s="27"/>
@@ -4070,7 +4070,7 @@
         <v>405</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F17" s="27"/>
       <c r="G17" s="27"/>
@@ -4114,7 +4114,7 @@
         <v>410</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F19" s="27"/>
       <c r="G19" s="27"/>
@@ -4158,7 +4158,7 @@
         <v>413</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F21" s="27"/>
       <c r="G21" s="27"/>
@@ -4180,7 +4180,7 @@
         <v>416</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F22" s="27"/>
       <c r="G22" s="27"/>
@@ -4202,7 +4202,7 @@
         <v>418</v>
       </c>
       <c r="E23" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F23" s="27"/>
       <c r="G23" s="27"/>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="D28" s="27"/>
       <c r="E28" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F28" s="27"/>
       <c r="G28" s="27"/>
@@ -4374,7 +4374,7 @@
         <v>405</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F31" s="27"/>
       <c r="G31" s="27"/>
@@ -4418,7 +4418,7 @@
         <v>410</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F33" s="27"/>
       <c r="G33" s="27"/>
@@ -4462,7 +4462,7 @@
         <v>413</v>
       </c>
       <c r="E35" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F35" s="27"/>
       <c r="G35" s="27"/>
@@ -4484,7 +4484,7 @@
         <v>416</v>
       </c>
       <c r="E36" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F36" s="27"/>
       <c r="G36" s="27"/>
@@ -4506,7 +4506,7 @@
         <v>418</v>
       </c>
       <c r="E37" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F37" s="27"/>
       <c r="G37" s="27"/>
@@ -4594,7 +4594,7 @@
         <v>263</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F41" s="27"/>
       <c r="G41" s="27"/>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="D46" s="27"/>
       <c r="E46" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F46" s="27"/>
       <c r="G46" s="27"/>
@@ -4766,7 +4766,7 @@
         <v>405</v>
       </c>
       <c r="E49" s="27" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F49" s="27"/>
       <c r="G49" s="27"/>
@@ -4810,7 +4810,7 @@
         <v>410</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F51" s="27"/>
       <c r="G51" s="27"/>
@@ -4854,7 +4854,7 @@
         <v>413</v>
       </c>
       <c r="E53" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F53" s="27"/>
       <c r="G53" s="27"/>
@@ -4876,7 +4876,7 @@
         <v>416</v>
       </c>
       <c r="E54" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F54" s="27"/>
       <c r="G54" s="27"/>
@@ -4898,7 +4898,7 @@
         <v>418</v>
       </c>
       <c r="E55" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F55" s="27"/>
       <c r="G55" s="27"/>
@@ -4947,7 +4947,7 @@
       <c r="F57" s="27"/>
       <c r="G57" s="27"/>
       <c r="H57" s="27" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="D63" s="27"/>
       <c r="E63" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F63" s="27"/>
       <c r="G63" s="27"/>
@@ -5136,7 +5136,7 @@
         <v>405</v>
       </c>
       <c r="E66" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F66" s="27"/>
       <c r="G66" s="27"/>
@@ -5180,7 +5180,7 @@
         <v>410</v>
       </c>
       <c r="E68" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F68" s="27"/>
       <c r="G68" s="27"/>
@@ -5224,7 +5224,7 @@
         <v>413</v>
       </c>
       <c r="E70" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F70" s="27"/>
       <c r="G70" s="27"/>
@@ -5246,7 +5246,7 @@
         <v>416</v>
       </c>
       <c r="E71" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F71" s="27"/>
       <c r="G71" s="27"/>
@@ -5268,7 +5268,7 @@
         <v>418</v>
       </c>
       <c r="E72" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F72" s="27"/>
       <c r="G72" s="27"/>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="D76" s="27"/>
       <c r="E76" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F76" s="27"/>
       <c r="G76" s="27"/>
@@ -5418,7 +5418,7 @@
         <v>405</v>
       </c>
       <c r="E79" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F79" s="27"/>
       <c r="G79" s="27"/>
@@ -5462,7 +5462,7 @@
         <v>410</v>
       </c>
       <c r="E81" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F81" s="27"/>
       <c r="G81" s="27"/>
@@ -5506,7 +5506,7 @@
         <v>413</v>
       </c>
       <c r="E83" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F83" s="27"/>
       <c r="G83" s="27"/>
@@ -5528,7 +5528,7 @@
         <v>416</v>
       </c>
       <c r="E84" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F84" s="27"/>
       <c r="G84" s="27"/>
@@ -5550,7 +5550,7 @@
         <v>418</v>
       </c>
       <c r="E85" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F85" s="27"/>
       <c r="G85" s="27"/>
@@ -5594,7 +5594,7 @@
         <v>285</v>
       </c>
       <c r="E87" s="27" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F87" s="27"/>
       <c r="G87" s="27"/>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="D90" s="27"/>
       <c r="E90" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F90" s="27"/>
       <c r="G90" s="27"/>
@@ -5722,7 +5722,7 @@
         <v>405</v>
       </c>
       <c r="E93" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F93" s="27"/>
       <c r="G93" s="27"/>
@@ -5766,7 +5766,7 @@
         <v>410</v>
       </c>
       <c r="E95" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F95" s="27"/>
       <c r="G95" s="27"/>
@@ -5810,7 +5810,7 @@
         <v>413</v>
       </c>
       <c r="E97" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F97" s="27"/>
       <c r="G97" s="27"/>
@@ -5832,7 +5832,7 @@
         <v>416</v>
       </c>
       <c r="E98" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F98" s="27"/>
       <c r="G98" s="27"/>
@@ -5854,7 +5854,7 @@
         <v>418</v>
       </c>
       <c r="E99" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F99" s="27"/>
       <c r="G99" s="27"/>
@@ -5898,7 +5898,7 @@
         <v>285</v>
       </c>
       <c r="E101" s="27" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F101" s="27"/>
       <c r="G101" s="27"/>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="D104" s="27"/>
       <c r="E104" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F104" s="27"/>
       <c r="G104" s="27"/>
@@ -6026,7 +6026,7 @@
         <v>405</v>
       </c>
       <c r="E107" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F107" s="27"/>
       <c r="G107" s="27"/>
@@ -6070,7 +6070,7 @@
         <v>410</v>
       </c>
       <c r="E109" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F109" s="27"/>
       <c r="G109" s="27"/>
@@ -6114,7 +6114,7 @@
         <v>413</v>
       </c>
       <c r="E111" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F111" s="27"/>
       <c r="G111" s="27"/>
@@ -6136,7 +6136,7 @@
         <v>416</v>
       </c>
       <c r="E112" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F112" s="27"/>
       <c r="G112" s="27"/>
@@ -6158,7 +6158,7 @@
         <v>418</v>
       </c>
       <c r="E113" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F113" s="27"/>
       <c r="G113" s="27"/>
@@ -6202,7 +6202,7 @@
         <v>285</v>
       </c>
       <c r="E115" s="27" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F115" s="27"/>
       <c r="G115" s="27"/>
@@ -6268,7 +6268,7 @@
         <v>285</v>
       </c>
       <c r="E118" s="27" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F118" s="27"/>
       <c r="G118" s="27"/>
@@ -6334,7 +6334,7 @@
         <v>285</v>
       </c>
       <c r="E121" s="27" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F121" s="27"/>
       <c r="G121" s="27"/>
@@ -6400,7 +6400,7 @@
         <v>285</v>
       </c>
       <c r="E124" s="27" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F124" s="27"/>
       <c r="G124" s="27"/>
@@ -6466,7 +6466,7 @@
         <v>285</v>
       </c>
       <c r="E127" s="27" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F127" s="27"/>
       <c r="G127" s="27"/>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="D130" s="27"/>
       <c r="E130" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F130" s="27"/>
       <c r="G130" s="27"/>
@@ -6594,7 +6594,7 @@
         <v>405</v>
       </c>
       <c r="E133" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F133" s="27"/>
       <c r="G133" s="27"/>
@@ -6638,7 +6638,7 @@
         <v>410</v>
       </c>
       <c r="E135" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F135" s="27"/>
       <c r="G135" s="27"/>
@@ -6682,7 +6682,7 @@
         <v>413</v>
       </c>
       <c r="E137" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F137" s="27"/>
       <c r="G137" s="27"/>
@@ -6704,7 +6704,7 @@
         <v>416</v>
       </c>
       <c r="E138" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F138" s="27"/>
       <c r="G138" s="27"/>
@@ -6726,7 +6726,7 @@
         <v>418</v>
       </c>
       <c r="E139" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F139" s="27"/>
       <c r="G139" s="27"/>
@@ -6792,7 +6792,7 @@
         <v>432</v>
       </c>
       <c r="E142" s="27" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="F142" s="27"/>
       <c r="G142" s="27"/>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="D144" s="27"/>
       <c r="E144" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F144" s="27"/>
       <c r="G144" s="27"/>
@@ -6898,7 +6898,7 @@
         <v>405</v>
       </c>
       <c r="E147" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F147" s="27"/>
       <c r="G147" s="27"/>
@@ -6942,7 +6942,7 @@
         <v>410</v>
       </c>
       <c r="E149" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F149" s="27"/>
       <c r="G149" s="27"/>
@@ -6986,7 +6986,7 @@
         <v>413</v>
       </c>
       <c r="E151" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F151" s="27"/>
       <c r="G151" s="27"/>
@@ -7008,7 +7008,7 @@
         <v>416</v>
       </c>
       <c r="E152" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F152" s="27"/>
       <c r="G152" s="27"/>
@@ -7030,7 +7030,7 @@
         <v>418</v>
       </c>
       <c r="E153" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F153" s="27"/>
       <c r="G153" s="27"/>
@@ -7096,7 +7096,7 @@
         <v>432</v>
       </c>
       <c r="E156" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F156" s="27"/>
       <c r="G156" s="27"/>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="D159" s="27"/>
       <c r="E159" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F159" s="27"/>
       <c r="G159" s="27"/>
@@ -7224,7 +7224,7 @@
         <v>405</v>
       </c>
       <c r="E162" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F162" s="27"/>
       <c r="G162" s="27"/>
@@ -7268,7 +7268,7 @@
         <v>410</v>
       </c>
       <c r="E164" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F164" s="27"/>
       <c r="G164" s="27"/>
@@ -7312,7 +7312,7 @@
         <v>413</v>
       </c>
       <c r="E166" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F166" s="27"/>
       <c r="G166" s="27"/>
@@ -7334,7 +7334,7 @@
         <v>416</v>
       </c>
       <c r="E167" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F167" s="27"/>
       <c r="G167" s="27"/>
@@ -7356,7 +7356,7 @@
         <v>418</v>
       </c>
       <c r="E168" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F168" s="27"/>
       <c r="G168" s="27"/>
@@ -7422,7 +7422,7 @@
         <v>432</v>
       </c>
       <c r="E171" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F171" s="27"/>
       <c r="G171" s="27"/>
@@ -7488,7 +7488,7 @@
         <v>432</v>
       </c>
       <c r="E174" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F174" s="27"/>
       <c r="G174" s="27"/>
@@ -7554,7 +7554,7 @@
         <v>432</v>
       </c>
       <c r="E177" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F177" s="27"/>
       <c r="G177" s="27"/>
@@ -7620,7 +7620,7 @@
         <v>432</v>
       </c>
       <c r="E180" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F180" s="27"/>
       <c r="G180" s="27"/>
@@ -7686,7 +7686,7 @@
         <v>432</v>
       </c>
       <c r="E183" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F183" s="27"/>
       <c r="G183" s="27"/>
@@ -7752,7 +7752,7 @@
         <v>432</v>
       </c>
       <c r="E186" s="27" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F186" s="27"/>
       <c r="G186" s="27"/>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D188" s="27"/>
       <c r="E188" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F188" s="27"/>
       <c r="G188" s="27"/>
@@ -7858,7 +7858,7 @@
         <v>405</v>
       </c>
       <c r="E191" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F191" s="27"/>
       <c r="G191" s="27"/>
@@ -7902,7 +7902,7 @@
         <v>410</v>
       </c>
       <c r="E193" s="27" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F193" s="27"/>
       <c r="G193" s="27"/>
@@ -7946,7 +7946,7 @@
         <v>413</v>
       </c>
       <c r="E195" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F195" s="27"/>
       <c r="G195" s="27"/>
@@ -7968,7 +7968,7 @@
         <v>416</v>
       </c>
       <c r="E196" s="27" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F196" s="27"/>
       <c r="G196" s="27"/>
@@ -7990,7 +7990,7 @@
         <v>418</v>
       </c>
       <c r="E197" s="27">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F197" s="27"/>
       <c r="G197" s="27"/>
@@ -8078,7 +8078,7 @@
         <v>285</v>
       </c>
       <c r="E201" s="27" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F201" s="27"/>
       <c r="G201" s="27"/>
@@ -8543,7 +8543,7 @@
         <v>262</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
@@ -8554,7 +8554,7 @@
         <v>262</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="39.6" x14ac:dyDescent="0.3">
@@ -8565,7 +8565,7 @@
         <v>262</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
@@ -8576,7 +8576,7 @@
         <v>262</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -8587,7 +8587,7 @@
         <v>262</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>

</xml_diff>